<commit_message>
AI-audit-log Week 4 (slot1+2)
</commit_message>
<xml_diff>
--- a/AI Audit Log_NguyenHoanAnhQuan.xlsx
+++ b/AI Audit Log_NguyenHoanAnhQuan.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SUMMER2026\SWD392_SU26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D26BA4C5-0218-4770-9EFE-9EED970EDF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8061E323-C529-41FF-8153-FA2E94473AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="3" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="5" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
     <sheet name="Week2" sheetId="2" r:id="rId2"/>
     <sheet name="Week3.1" sheetId="3" r:id="rId3"/>
     <sheet name="Week3.2" sheetId="5" r:id="rId4"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId5"/>
+    <sheet name="Week4.1" sheetId="6" r:id="rId5"/>
+    <sheet name="Week4.2" sheetId="7" r:id="rId6"/>
+    <sheet name="Assignment 3" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="129">
   <si>
     <t>Ví dụ: Abstraction</t>
   </si>
@@ -353,19 +355,185 @@
     <t>Phản hồi: AI kiểm tra các lỗi như thiếu multiplicity, sai quan hệ inheritance hoặc dùng sai composition/aggregation.
 Kiểm chứng: Tôi so sánh lại với slide UML và góp ý của giảng viên trên lớp.
 Quyết định: Chỉnh sửa sơ đồ theo góp ý để hoàn thiện bản cuối cùng nộp nhóm.</t>
+  </si>
+  <si>
+    <t>Xác định Class</t>
+  </si>
+  <si>
+    <t>"Đối với hệ thống Smart Queue Management System Using AI, các class chính nên gồm những gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất các class User, Queue, Ticket, ServiceCounter, QueuePredictionAI, Notification, Feedback.
+Kiểm chứng: Tôi đối chiếu với chức năng của hệ thống đã phân tích trước đó.
+Quyết định: Chọn các class phù hợp để xây dựng class diagram.</t>
+  </si>
+  <si>
+    <t>Entity Class</t>
+  </si>
+  <si>
+    <t>"Những class nào nên được đánh dấu là Entity Class?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI xác định User, Queue, Ticket, Appointment, Feedback là các entity class vì lưu trữ dữ liệu lâu dài.
+Kiểm chứng: So sánh với lý thuyết Entity Class trong slide.
+Quyết định: Áp dụng stereotype «entity» cho các class này.</t>
+  </si>
+  <si>
+    <t>Association</t>
+  </si>
+  <si>
+    <t>"Mối quan hệ giữa User và Ticket nên được mô hình hóa như thế nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất Association 1 User có thể sở hữu nhiều Ticket.
+Kiểm chứng: Đối chiếu với quy trình lấy số thứ tự của khách hàng.
+Quyết định: Sử dụng multiplicity 1..* trong sơ đồ.</t>
+  </si>
+  <si>
+    <t>"Multiplicity giữa Queue và Ticket là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: Một Queue chứa nhiều Ticket, mỗi Ticket chỉ thuộc một Queue.
+Kiểm chứng: Đúng với nghiệp vụ hàng chờ.
+Quyết định: Áp dụng 1..* giữa Queue và Ticket.</t>
+  </si>
+  <si>
+    <t>Composition</t>
+  </si>
+  <si>
+    <t>"Queue và Ticket nên dùng Association hay Composition?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất Composition vì Ticket không tồn tại nếu Queue bị xóa.
+Kiểm chứng: Đối chiếu với khái niệm Composition trong bài học.
+Quyết định: Dùng Composition trong UML.</t>
+  </si>
+  <si>
+    <t>"Có thể sử dụng kế thừa trong hệ thống này không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất User là superclass, Customer và Staff là subclasses.
+Kiểm chứng: Kiểm tra với chức năng của từng loại người dùng.
+Quyết định: Áp dụng Generalization/Specialization.</t>
+  </si>
+  <si>
+    <t>Kiểm tra UML</t>
+  </si>
+  <si>
+    <t>"Class Diagram hiện tại có thiếu quan hệ nào không?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI phát hiện thiếu quan hệ giữa ServiceCounter và Queue.
+Kiểm chứng: Đối chiếu với luồng phục vụ khách hàng.
+Quyết định: Bổ sung quan hệ còn thiếu vào sơ đồ.</t>
+  </si>
+  <si>
+    <t>Dynamic Modeling</t>
+  </si>
+  <si>
+    <t>"Dynamic Modeling là gì trong UML?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Dynamic Modeling mô tả hành vi động của hệ thống, tập trung vào luồng điều khiển và tương tác giữa các đối tượng theo thời gian.
+Kiểm chứng: Tôi đối chiếu với slide Ch09-11 và thấy phù hợp với định nghĩa của bài học.
+Quyết định: Sử dụng khái niệm này để phân biệt với Static Modeling đã học trước đó.</t>
+  </si>
+  <si>
+    <t>Dynamic Interaction Modeling</t>
+  </si>
+  <si>
+    <t>"Dynamic Interaction Modeling dùng để làm gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho biết Dynamic Interaction Modeling được sử dụng để mô tả cách các object tương tác nhằm hiện thực hóa Use Case.
+Kiểm chứng: Tôi đối chiếu với phần Dynamic Interaction Modeling trong slide.
+Quyết định: Áp dụng khi phân tích các Use Case của dự án nhóm.</t>
+  </si>
+  <si>
+    <t>Communication Diagram</t>
+  </si>
+  <si>
+    <t>"Communication Diagram là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đây là sơ đồ UML mô tả sự tương tác giữa các object thông qua các message và số thứ tự message.
+Kiểm chứng: Tôi đối chiếu với định nghĩa trong slide.
+Quyết định: Sử dụng Communication Diagram để mô tả tương tác trong hệ thống.</t>
+  </si>
+  <si>
+    <t>Sequence Diagram</t>
+  </si>
+  <si>
+    <t>"Sequence Diagram là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích Sequence Diagram thể hiện thứ tự gửi nhận message giữa các object theo thời gian từ trên xuống dưới.
+Kiểm chứng: So sánh với ví dụ View Alarms trong slide.
+Quyết định: Dùng Sequence Diagram để mô tả luồng xử lý chính của hệ thống.</t>
+  </si>
+  <si>
+    <t>Sequence vs Communication</t>
+  </si>
+  <si>
+    <t>"Sự khác nhau giữa Sequence Diagram và Communication Diagram?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI cho biết Sequence Diagram nhấn mạnh yếu tố thời gian còn Communication Diagram nhấn mạnh mối liên kết giữa các object.
+Kiểm chứng: Đối chiếu với bảng so sánh trong slide.
+Quyết định: Hiểu ưu điểm của từng loại sơ đồ để sử dụng phù hợp.</t>
+  </si>
+  <si>
+    <t>UC Realization</t>
+  </si>
+  <si>
+    <t>"Làm thế nào để xây dựng Sequence Diagram từ Use Case?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI đề xuất xác định actor, boundary object, control object và message sequence.
+Kiểm chứng: So sánh với quy trình trong bài học.
+Quyết định: Áp dụng cho Use Case của dự án Smart Queue Management System.</t>
+  </si>
+  <si>
+    <t>Main Scenario</t>
+  </si>
+  <si>
+    <t>"Main Sequence trong Dynamic Modeling là gì?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đây là luồng xử lý chính của Use Case khi mọi điều kiện đều thành công.
+Kiểm chứng: Đối chiếu với ví dụ Make Order Request.
+Quyết định: Sử dụng để xây dựng Sequence Diagram chính.</t>
+  </si>
+  <si>
+    <t>Alternative Scenario</t>
+  </si>
+  <si>
+    <t>"Alternative Sequence được biểu diễn như thế nào?"</t>
+  </si>
+  <si>
+    <t>Phản hồi: AI giải thích đây là các luồng xử lý thay thế khi có ngoại lệ hoặc điều kiện khác xảy ra.
+Kiểm chứng: So sánh với trường hợp Credit Card Denied trong slide.
+Quyết định: Bổ sung các nhánh thay thế vào Sequence Diagram.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="163"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -412,7 +580,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -426,7 +594,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -434,6 +602,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -773,15 +953,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBDDC7E-59F2-4CBB-B3D2-F6FB78F9E873}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="20.9375" customWidth="1"/>
-    <col min="2" max="2" width="26.875" customWidth="1"/>
-    <col min="3" max="3" width="24.25" customWidth="1"/>
+    <col min="1" max="1" width="20.9296875" customWidth="1"/>
+    <col min="2" max="2" width="26.86328125" customWidth="1"/>
+    <col min="3" max="3" width="24.265625" customWidth="1"/>
     <col min="4" max="4" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="13.9">
+    <row r="1" spans="1:5">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -796,7 +976,7 @@
       </c>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="67.5">
+    <row r="2" spans="1:5" ht="71.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -810,7 +990,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="54">
+    <row r="3" spans="1:5" ht="57">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -824,7 +1004,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="67.5">
+    <row r="4" spans="1:5" ht="71.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -838,7 +1018,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="81">
+    <row r="5" spans="1:5" ht="85.5">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -860,14 +1040,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59E3EFE9-6FFB-49CC-BE69-0C0E36C6253E}">
   <dimension ref="A1:D32"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="41.9375" customWidth="1"/>
-    <col min="3" max="3" width="45.8125" customWidth="1"/>
-    <col min="4" max="4" width="44.875" customWidth="1"/>
+    <col min="2" max="2" width="41.9296875" customWidth="1"/>
+    <col min="3" max="3" width="45.796875" customWidth="1"/>
+    <col min="4" max="4" width="44.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="27.75">
+    <row r="1" spans="1:4" ht="28.5">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -1018,9 +1198,9 @@
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="47.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="22.875" customWidth="1"/>
-    <col min="3" max="3" width="54.3125" customWidth="1"/>
-    <col min="4" max="4" width="77.5" customWidth="1"/>
+    <col min="2" max="2" width="22.86328125" customWidth="1"/>
+    <col min="3" max="3" width="54.33203125" customWidth="1"/>
+    <col min="4" max="4" width="77.46484375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="47.75" customHeight="1">
@@ -1213,15 +1393,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C2795E5-0A07-4918-BFC6-ED555F7A394E}">
   <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="8.9375" customWidth="1"/>
-    <col min="2" max="2" width="32.5" customWidth="1"/>
-    <col min="3" max="3" width="26.375" customWidth="1"/>
-    <col min="4" max="4" width="58.8125" customWidth="1"/>
+    <col min="1" max="1" width="8.9296875" customWidth="1"/>
+    <col min="2" max="2" width="32.46484375" customWidth="1"/>
+    <col min="3" max="3" width="26.3984375" customWidth="1"/>
+    <col min="4" max="4" width="58.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="13.9">
+    <row r="1" spans="1:4">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -1332,9 +1512,291 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65D2BBFF-A5A9-4621-A1B0-B5B41A144524}">
+  <dimension ref="A1:D29"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="9.19921875" customWidth="1"/>
+    <col min="2" max="2" width="34.06640625" customWidth="1"/>
+    <col min="3" max="3" width="41.796875" customWidth="1"/>
+    <col min="4" max="4" width="47.53125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="118.25" customHeight="1">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="134.35" customHeight="1">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="96.4" customHeight="1">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="96.4" customHeight="1">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="96.4" customHeight="1">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="96.4" customHeight="1">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="96.4" customHeight="1">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" ht="12.75" customHeight="1"/>
+    <row r="18" hidden="1"/>
+    <row r="19" hidden="1"/>
+    <row r="20" hidden="1"/>
+    <row r="21" hidden="1"/>
+    <row r="22" hidden="1"/>
+    <row r="23" hidden="1"/>
+    <row r="24" hidden="1"/>
+    <row r="25" hidden="1"/>
+    <row r="26" hidden="1"/>
+    <row r="27" hidden="1"/>
+    <row r="28" hidden="1"/>
+    <row r="29" hidden="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{966BDC56-E696-48BC-BCCD-FDFD9FA85D73}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="36.33203125" customWidth="1"/>
+    <col min="3" max="3" width="30.3984375" customWidth="1"/>
+    <col min="4" max="4" width="44.59765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="107.65" customHeight="1">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="108.75" customHeight="1">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="118.5" customHeight="1">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="99.4" customHeight="1">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="113.25" customHeight="1">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="97.5" customHeight="1">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="88.5" customHeight="1">
+      <c r="A8" s="12">
+        <v>7</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="103.9" customHeight="1">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>